<commit_message>
Qualitative picker: intro copy in the maintainer's voice
The first intro read unclear and not in her register, so the headline,
lead and header subtitle were re-offered and picked: concrete members
unpacked inline, the mechanism in the sentence, no shorthand. The
Teaching card mirrors the new lead's premise sentence, and the thumbnail
is retaken because it is a header screenshot that carries the headline.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0191t4cG3m6aQycW3EiNAUvs
</commit_message>
<xml_diff>
--- a/qualpicker/data/qualitative_displays.xlsx
+++ b/qualpicker/data/qualitative_displays.xlsx
@@ -4160,7 +4160,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Match the figure to what your coding produced and what you need it to show.</t>
+          <t>Match the figure to what your coding produced and how many cases you have.</t>
         </is>
       </c>
     </row>
@@ -4184,7 +4184,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>The memo is not the only way to show what the documents say.</t>
+          <t>Once interviews, statutes, or case files have been coded, they can be charted, and the chart depends on what the coding produced.</t>
         </is>
       </c>
     </row>
@@ -4196,7 +4196,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Coding turns documents and interviews into evidence with a shape: counts across cases, thresholds inside the text, stages, ties, or the passages themselves, and the figure that suits one shape misleads with another. Answer up to six questions about what you have, and every display sorts into what fits, what could fit with more cases or the text beside it, and what is the wrong tool here.</t>
+          <t>The same coded interviews can become a ranked bar chart, a matrix of cases by themes, a timeline, or a page of quotations, and which one is honest depends on what the coding produced, how many cases there are, and whether a count from those cases would mean anything. Answer up to six questions about what you have and every display sorts into what fits, what could fit with more cases or with the text beside it, and what is the wrong tool here.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Qualitative picker: tighten rule cells the first real test exposed
An in-list cell is an OR, so forms that need a process or a sequence
and counts were passing on counts alone (funnel, part-in-whole bars,
quote cards), and forms that need a sequence or a number were passing
on an Attributes they did not require (time-ordered matrix, spans over
time, span chart). Each now lists only the shape it cannot do without.
"Helpful, but not required" no longer fails pattern charts; only "the
quotes carry the evidence" earns the pair-with-the-text tag.

Found by running the maintainer's Missouri action plans (45 circuits,
41 categories) through the live page; the dataset stays off the repo.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0191t4cG3m6aQycW3EiNAUvs
</commit_message>
<xml_diff>
--- a/qualpicker/data/qualitative_displays.xlsx
+++ b/qualpicker/data/qualitative_displays.xlsx
@@ -1737,7 +1737,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Helpful;Pattern</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -1809,7 +1809,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Helpful;Pattern</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -1968,7 +1968,7 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Helpful;Pattern</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -2030,12 +2030,12 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Counts;Sequence</t>
+          <t>Sequence</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Happened;Common</t>
+          <t>Happened</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -2050,7 +2050,7 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Helpful;Pattern</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -2132,7 +2132,7 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Helpful;Pattern</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
@@ -2189,12 +2189,12 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Process;Counts</t>
+          <t>Process</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Branch;Common</t>
+          <t>Branch</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -2209,7 +2209,7 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Helpful;Pattern</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
@@ -2291,7 +2291,7 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Helpful;Pattern</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
@@ -2358,7 +2358,7 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Helpful;Pattern</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
@@ -2539,7 +2539,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Sequence;Attributes</t>
+          <t>Sequence</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -2601,7 +2601,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Attributes;Words</t>
+          <t>Words</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -2683,7 +2683,7 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Helpful;Pattern</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
@@ -2797,7 +2797,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Number;Attributes</t>
+          <t>Number</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -2817,7 +2817,7 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Helpful;Pattern</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
@@ -2899,7 +2899,7 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Helpful;Pattern</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
@@ -2981,7 +2981,7 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Helpful;Pattern</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
@@ -3120,7 +3120,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Sequence;Attributes</t>
+          <t>Sequence</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -3140,7 +3140,7 @@
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Helpful;Pattern</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
@@ -3656,12 +3656,12 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Words;Counts</t>
+          <t>Words</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Said;Common</t>
+          <t>Said</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">

</xml_diff>

<commit_message>
Qualitative picker: add the choropleth map and a Places answer
The first real test (Missouri circuit action plans) ended in a map
question: circuits are whole counties plus St. Louis City, so the count
heatmap can sit on a county map, and the picker had no row that could say
so. The shape axis gains a Places level and a new Places and maps family
holds one display, the choropleth, with a not_for about reading size
from area. Cartographic sources are flagged as still to come.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0191t4cG3m6aQycW3EiNAUvs
</commit_message>
<xml_diff>
--- a/qualpicker/data/qualitative_displays.xlsx
+++ b/qualpicker/data/qualitative_displays.xlsx
@@ -698,7 +698,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D30"/>
+  <dimension ref="A1:D31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -786,7 +786,7 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="5">
@@ -806,7 +806,7 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="6">
@@ -826,7 +826,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="7">
@@ -846,7 +846,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="8">
@@ -866,7 +866,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="9">
@@ -886,7 +886,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="10">
@@ -1306,6 +1306,26 @@
         </is>
       </c>
       <c r="D30" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>shape</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Places</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Places on a map (a value or feature per county, circuit, or state)</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
         <v>3</v>
       </c>
     </row>
@@ -1320,7 +1340,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U38"/>
+  <dimension ref="A1:U39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -4122,6 +4142,77 @@
         </is>
       </c>
     </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>CHORO</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Choropleth map (shaded areas)</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Places and maps</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Each place on its own outline, shaded by a value or marked for a feature.</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Places</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>Compare;Common</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>Handful</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr"/>
+      <c r="I39" t="inlineStr"/>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>Helpful;Pattern</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr"/>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>Pattern</t>
+        </is>
+      </c>
+      <c r="M39" t="inlineStr">
+        <is>
+          <t>Cases that are places, when where a feature sits is part of the finding: which circuits named transportation, which states require a diagnosis, one map per feature if there are several.</t>
+        </is>
+      </c>
+      <c r="N39" t="inlineStr">
+        <is>
+          <t>Reading size from area. Large rural units fill the eye while a city of a million is a speck, so label the small ones, add an inset, or let the map carry the geography and a heatmap carry the comparison.</t>
+        </is>
+      </c>
+      <c r="O39" t="inlineStr"/>
+      <c r="P39" t="inlineStr"/>
+      <c r="Q39" t="inlineStr">
+        <is>
+          <t>Chart form in common use, the thematic map's workhorse; cartographic sources to follow the visualization-literature rescan.</t>
+        </is>
+      </c>
+      <c r="R39" t="inlineStr"/>
+      <c r="S39" t="inlineStr"/>
+      <c r="T39" t="inlineStr"/>
+      <c r="U39" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Qualitative picker: add the pictograph row
The icon array (one mark per case) was already in; the pictograph is the
other icon form, one icon per set number of cases, so it needs a round
unit: a few dozen cases at least, a defensible count, and a not_for about
half icons and too many categories. Infographics stay in the format
picker as a deliverable.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0191t4cG3m6aQycW3EiNAUvs
</commit_message>
<xml_diff>
--- a/qualpicker/data/qualitative_displays.xlsx
+++ b/qualpicker/data/qualitative_displays.xlsx
@@ -1340,7 +1340,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U39"/>
+  <dimension ref="A1:U40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1717,12 +1717,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>WAFFLE</t>
+          <t>PICTO</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Dot matrix (waffle)</t>
+          <t>Pictograph (icon units)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -1732,7 +1732,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>A hundred squares, some filled: a share shown as a grid rather than a pie.</t>
+          <t>A row of icons per category, each icon standing for a set number of cases, so the bar is also a tally.</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -1742,12 +1742,12 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Common</t>
+          <t>Common;Compare</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Many</t>
+          <t>Dozens</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -1772,29 +1772,29 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>A single share from a large population, read as 'so many in a hundred'.</t>
+          <t>A few categories whose counts are large and round enough that one icon can stand for ten or a hundred cases, for a reader who will not read an axis.</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>More than three or four categories, or a count so small that each square stands for a person you could name.</t>
+          <t>Counts that do not divide evenly, because a half icon reads as half a case, and more than five or six categories, where the rows stop being countable.</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>Chart form in common use.</t>
+          <t>Chart form in common use (the Isotype unit chart); perception sources to follow the visualization-literature rescan.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>PIE</t>
+          <t>WAFFLE</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Pie chart</t>
+          <t>Dot matrix (waffle)</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -1804,7 +1804,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>A circle cut into shares. Kept here so the page can say when it works, which is rarely.</t>
+          <t>A hundred squares, some filled: a share shown as a grid rather than a pie.</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -1834,7 +1834,7 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>One</t>
+          <t>One;Two</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -1844,34 +1844,29 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>One share against the rest, when the share is far from half and there is only one pie.</t>
+          <t>A single share from a large population, read as 'so many in a hundred'.</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>More than three slices, any two slices of similar size, two pies side by side, or anything a bar would show more exactly.</t>
+          <t>More than three or four categories, or a count so small that each square stands for a person you could name.</t>
         </is>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
           <t>Chart form in common use.</t>
-        </is>
-      </c>
-      <c r="U6" t="inlineStr">
-        <is>
-          <t>A pie of {have} is a pie of three or four people; a bar shows the same counts without pretending they add to a whole.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>TILES</t>
+          <t>PIE</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Stat tiles</t>
+          <t>Pie chart</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -1881,12 +1876,12 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>A few big numbers with a line of context under each.</t>
+          <t>A circle cut into shares. Kept here so the page can say when it works, which is rarely.</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Counts;Number</t>
+          <t>Counts</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -1896,7 +1891,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Handful</t>
+          <t>Many</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -1921,39 +1916,34 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>Three or four headline figures that need no comparison between them.</t>
+          <t>One share against the rest, when the share is far from half and there is only one pie.</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>Anything with a trend or a distribution behind it; a tile hides both.</t>
-        </is>
-      </c>
-      <c r="O7" t="inlineStr">
-        <is>
-          <t>A Right That Exists on Paper, Exhibit 06</t>
-        </is>
-      </c>
-      <c r="P7" t="inlineStr">
-        <is>
-          <t>../compassionaterelease/index.html#does-anyone-have-to-count</t>
+          <t>More than three slices, any two slices of similar size, two pies side by side, or anything a bar would show more exactly.</t>
         </is>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>Chart form in common use; the example links to where this site uses it.</t>
+          <t>Chart form in common use.</t>
+        </is>
+      </c>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>A pie of {have} is a pie of three or four people; a bar shows the same counts without pretending they add to a whole.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>MULT</t>
+          <t>TILES</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Small multiples</t>
+          <t>Stat tiles</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -1963,22 +1953,22 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>The same small chart repeated once per group on one scale, so the eye compares panels.</t>
+          <t>A few big numbers with a line of context under each.</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Counts;Sequence;Number</t>
+          <t>Counts;Number</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Compare;Happened</t>
+          <t>Common</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Dozens</t>
+          <t>Handful</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -1993,7 +1983,7 @@
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>Two;Several</t>
+          <t>One</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
@@ -2003,22 +1993,22 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>Comparing several groups on the same measure without stacking them into one crowded panel.</t>
+          <t>Three or four headline figures that need no comparison between them.</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>One group, or panels so different in scale that a shared axis flattens half of them.</t>
+          <t>Anything with a trend or a distribution behind it; a tile hides both.</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>A Right That Exists on Paper, Exhibit 08</t>
+          <t>A Right That Exists on Paper, Exhibit 06</t>
         </is>
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>../compassionaterelease/index.html#why-courts-say-yes-and-why-they-say-no</t>
+          <t>../compassionaterelease/index.html#does-anyone-have-to-count</t>
         </is>
       </c>
       <c r="Q8" t="inlineStr">
@@ -2030,12 +2020,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>MONTH</t>
+          <t>MULT</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Part-in-whole bars over time</t>
+          <t>Small multiples</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -2045,17 +2035,17 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Monthly or yearly totals with the part of interest filled, so the share and the trend show together.</t>
+          <t>The same small chart repeated once per group on one scale, so the eye compares panels.</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Sequence</t>
+          <t>Counts;Sequence;Number</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Happened</t>
+          <t>Compare;Happened</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -2075,7 +2065,7 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>One;Two</t>
+          <t>Two;Several</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
@@ -2085,22 +2075,22 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>A docket or caseload over time where one outcome (granted, released) is a slice of each period's total.</t>
+          <t>Comparing several groups on the same measure without stacking them into one crowded panel.</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>More than two parts, or periods with counts too small to shade.</t>
+          <t>One group, or panels so different in scale that a shared axis flattens half of them.</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>A Right That Exists on Paper, Exhibit 07</t>
+          <t>A Right That Exists on Paper, Exhibit 08</t>
         </is>
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>../compassionaterelease/index.html#the-federal-docket</t>
+          <t>../compassionaterelease/index.html#why-courts-say-yes-and-why-they-say-no</t>
         </is>
       </c>
       <c r="Q9" t="inlineStr">
@@ -2112,12 +2102,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>HEAT</t>
+          <t>MONTH</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Count heatmap</t>
+          <t>Part-in-whole bars over time</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -2127,17 +2117,17 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Cases down the side, codes across the top, each cell shaded by how many.</t>
+          <t>Monthly or yearly totals with the part of interest filled, so the share and the trend show together.</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Counts;Attributes;Relationships</t>
+          <t>Sequence</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Compare;Together</t>
+          <t>Happened</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -2155,6 +2145,11 @@
           <t>Helpful;Pattern</t>
         </is>
       </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>One;Two</t>
+        </is>
+      </c>
       <c r="L10" t="inlineStr">
         <is>
           <t>Pattern</t>
@@ -2162,39 +2157,39 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>Seeing which codes cluster in which cases when both lists are long.</t>
+          <t>A docket or caseload over time where one outcome (granted, released) is a slice of each period's total.</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>Exact values; shading is for pattern, and a reader who needs the number needs a table.</t>
+          <t>More than two parts, or periods with counts too small to shade.</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>Maturity Gap, The Spread Inside Every Age</t>
+          <t>A Right That Exists on Paper, Exhibit 07</t>
         </is>
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>../countedwrong/index.html#the-spread-inside-every-age</t>
+          <t>../compassionaterelease/index.html#the-federal-docket</t>
         </is>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>Henderson and Segal (2013) shade a theme-by-case matrix by importance (their Figure 3.5); the example links to where this site uses the form.</t>
+          <t>Chart form in common use; the example links to where this site uses it.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>FUNNEL</t>
+          <t>HEAT</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Nested-bar funnel</t>
+          <t>Count heatmap</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -2204,17 +2199,17 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Each stage drawn inside the one before it, so the drop-off is the shape.</t>
+          <t>Cases down the side, codes across the top, each cell shaded by how many.</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Process</t>
+          <t>Counts;Attributes;Relationships</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Branch</t>
+          <t>Compare;Together</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -2232,11 +2227,6 @@
           <t>Helpful;Pattern</t>
         </is>
       </c>
-      <c r="K11" t="inlineStr">
-        <is>
-          <t>One;Two</t>
-        </is>
-      </c>
       <c r="L11" t="inlineStr">
         <is>
           <t>Pattern</t>
@@ -2244,39 +2234,39 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>Attrition through a fixed sequence of stages: eligible to applied to granted.</t>
+          <t>Seeing which codes cluster in which cases when both lists are long.</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>Stages that are not nested, where a case can enter late or skip one.</t>
+          <t>Exact values; shading is for pattern, and a reader who needs the number needs a table.</t>
         </is>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>A Right That Exists on Paper, Exhibit 05</t>
+          <t>Maturity Gap, The Spread Inside Every Age</t>
         </is>
       </c>
       <c r="P11" t="inlineStr">
         <is>
-          <t>../compassionaterelease/index.html#eligible-applied-released</t>
+          <t>../countedwrong/index.html#the-spread-inside-every-age</t>
         </is>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>Chart form in common use; the example links to where this site uses it.</t>
+          <t>Henderson and Segal (2013) shade a theme-by-case matrix by importance (their Figure 3.5); the example links to where this site uses the form.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>ALLUV</t>
+          <t>FUNNEL</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Alluvial (flows between stages)</t>
+          <t>Nested-bar funnel</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -2286,17 +2276,17 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Ribbons that carry cases from one stage's categories to the next stage's.</t>
+          <t>Each stage drawn inside the one before it, so the drop-off is the shape.</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Process;Relationships</t>
+          <t>Process</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Branch;Together</t>
+          <t>Branch</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -2314,6 +2304,11 @@
           <t>Helpful;Pattern</t>
         </is>
       </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>One;Two</t>
+        </is>
+      </c>
       <c r="L12" t="inlineStr">
         <is>
           <t>Pattern</t>
@@ -2321,29 +2316,39 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>How cases move between categories over two or three stages, such as reason given to outcome reached.</t>
+          <t>Attrition through a fixed sequence of stages: eligible to applied to granted.</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>More than three stages or many categories, where the ribbons tangle, or a reader who needs the counts.</t>
+          <t>Stages that are not nested, where a case can enter late or skip one.</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>A Right That Exists on Paper, Exhibit 05</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>../compassionaterelease/index.html#eligible-applied-released</t>
         </is>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
-          <t>Chart form in common use.</t>
+          <t>Chart form in common use; the example links to where this site uses it.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>TREEMAP</t>
+          <t>ALLUV</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Treemap</t>
+          <t>Alluvial (flows between stages)</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -2353,17 +2358,17 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Nested rectangles sized by count, themes holding their subthemes.</t>
+          <t>Ribbons that carry cases from one stage's categories to the next stage's.</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Nested;Counts</t>
+          <t>Process;Relationships</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Organised;Common</t>
+          <t>Branch;Together</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -2381,11 +2386,6 @@
           <t>Helpful;Pattern</t>
         </is>
       </c>
-      <c r="K13" t="inlineStr">
-        <is>
-          <t>One</t>
-        </is>
-      </c>
       <c r="L13" t="inlineStr">
         <is>
           <t>Pattern</t>
@@ -2393,12 +2393,12 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>A coding hierarchy where the sizes matter and the hierarchy is shallow.</t>
+          <t>How cases move between categories over two or three stages, such as reason given to outcome reached.</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>Comparing sizes precisely, or a hierarchy more than two levels deep.</t>
+          <t>More than three stages or many categories, where the ribbons tangle, or a reader who needs the counts.</t>
         </is>
       </c>
       <c r="Q13" t="inlineStr">
@@ -2410,74 +2410,84 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>FRAME</t>
+          <t>TREEMAP</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Framework matrix</t>
+          <t>Treemap</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Matrices</t>
+          <t>Counting the codes</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Cases down the side, themes across, and in each cell a summary of what that case said about that theme.</t>
+          <t>Nested rectangles sized by count, themes holding their subthemes.</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Attributes;Words</t>
+          <t>Nested;Counts</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Compare;Said</t>
+          <t>Organised;Common</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Handful</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
           <t>Dozens</t>
         </is>
       </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Census;Designed</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Helpful;Pattern</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>One</t>
+        </is>
+      </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>Passages</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>Holding a whole qualitative dataset in one view, so cases can be compared theme by theme without losing the words.</t>
+          <t>A coding hierarchy where the sizes matter and the hierarchy is shallow.</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>A public audience or a slide; it is an analyst's instrument and a report appendix, not a figure.</t>
+          <t>Comparing sizes precisely, or a hierarchy more than two levels deep.</t>
         </is>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>Gale and colleagues (2013), the framework method; the matrix is the most common display in Verdinelli and Scagnoli's (2013) review.</t>
+          <t>Chart form in common use.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>CHECK</t>
+          <t>FRAME</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Presence-or-absence grid</t>
+          <t>Framework matrix</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -2487,17 +2497,17 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>A checkerboard: each case, each feature, a mark where it applies.</t>
+          <t>Cases down the side, themes across, and in each cell a summary of what that case said about that theme.</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Attributes</t>
+          <t>Attributes;Words</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Compare;Common</t>
+          <t>Compare;Said</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -2507,44 +2517,39 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>Many</t>
-        </is>
-      </c>
-      <c r="J15" t="inlineStr">
-        <is>
-          <t>Helpful;Pattern</t>
+          <t>Dozens</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Passages</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>Fifty statutes against a dozen provisions, where readers want to find their own state and read across.</t>
+          <t>Holding a whole qualitative dataset in one view, so cases can be compared theme by theme without losing the words.</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>Degrees: a mark is yes or no, and a feature that is partly present needs a different cell.</t>
+          <t>A public audience or a slide; it is an analyst's instrument and a report appendix, not a figure.</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>Miles, Huberman and Saldana, Qualitative Data Analysis: A Methods Sourcebook (the checklist matrix, among the methods of ordering a matrix).</t>
+          <t>Gale and colleagues (2013), the framework method; the matrix is the most common display in Verdinelli and Scagnoli's (2013) review.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>TIMEMAT</t>
+          <t>CHECK</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Time-ordered matrix</t>
+          <t>Presence-or-absence grid</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -2554,17 +2559,17 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Cases down the side, periods across, and what happened to each case in each period.</t>
+          <t>A checkerboard: each case, each feature, a mark where it applies.</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Sequence</t>
+          <t>Attributes</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Happened;Compare</t>
+          <t>Compare;Common</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -2574,39 +2579,44 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>Dozens</t>
+          <t>Many</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>Helpful;Pattern</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>Phrases</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>Several cases moving through the same periods, when the reader needs both the sequence and the comparison.</t>
+          <t>Fifty statutes against a dozen provisions, where readers want to find their own state and read across.</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>A single case (use a timeline) or exact dates (a matrix holds periods, not days).</t>
+          <t>Degrees: a mark is yes or no, and a feature that is partly present needs a different cell.</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>Miles, Huberman and Saldana, Qualitative Data Analysis: A Methods Sourcebook (matrix and network displays, and the methods of ordering them).</t>
+          <t>Miles, Huberman and Saldana, Qualitative Data Analysis: A Methods Sourcebook (the checklist matrix, among the methods of ordering a matrix).</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>ROLEMAT</t>
+          <t>TIMEMAT</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Role-ordered matrix</t>
+          <t>Time-ordered matrix</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -2616,17 +2626,17 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Rows are roles (judges, clerks, defendants), columns are themes, and cells are what each role said.</t>
+          <t>Cases down the side, periods across, and what happened to each case in each period.</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Words</t>
+          <t>Sequence</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Compare;Said</t>
+          <t>Happened;Compare</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -2641,17 +2651,17 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>Passages</t>
+          <t>Phrases</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>Showing that the same program looks different from different seats.</t>
+          <t>Several cases moving through the same periods, when the reader needs both the sequence and the comparison.</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>Roles with one informant each, where the row is a person rather than a role.</t>
+          <t>A single case (use a timeline) or exact dates (a matrix holds periods, not days).</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
@@ -2663,12 +2673,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>COOC</t>
+          <t>ROLEMAT</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Code co-occurrence matrix</t>
+          <t>Role-ordered matrix</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -2678,64 +2688,59 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Codes against codes, each cell counting how often two were applied to the same passage.</t>
+          <t>Rows are roles (judges, clerks, defendants), columns are themes, and cells are what each role said.</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Relationships;Counts</t>
+          <t>Words</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Together</t>
+          <t>Compare;Said</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
+          <t>Handful</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
           <t>Dozens</t>
         </is>
       </c>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>Census;Designed</t>
-        </is>
-      </c>
-      <c r="J18" t="inlineStr">
-        <is>
-          <t>Helpful;Pattern</t>
-        </is>
-      </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Passages</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>Finding which themes travel together across a large coded corpus.</t>
+          <t>Showing that the same program looks different from different seats.</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>Small datasets, where a co-occurrence of two or three means nothing, and any reading of cause.</t>
+          <t>Roles with one informant each, where the row is a person rather than a role.</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>Counting coded themes is what Onwuegbuzie and Dickinson (2008) call quantitizing; their crossover displays chart the result.</t>
+          <t>Miles, Huberman and Saldana, Qualitative Data Analysis: A Methods Sourcebook (matrix and network displays, and the methods of ordering them).</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>CODEBK</t>
+          <t>COOC</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Codebook table</t>
+          <t>Code co-occurrence matrix</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -2745,129 +2750,114 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Each code, its definition, and one passage that shows it.</t>
+          <t>Codes against codes, each cell counting how often two were applied to the same passage.</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Words;Nested</t>
+          <t>Relationships;Counts</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Organised;Said</t>
+          <t>Together</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>One</t>
+          <t>Dozens</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>Census;Designed</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>Helpful;Pattern</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>Passages</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>Making the coding auditable: a reader can check the rule against the example and argue with either.</t>
+          <t>Finding which themes travel together across a large coded corpus.</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>Findings; it defines the instrument and shows no result.</t>
-        </is>
-      </c>
-      <c r="O19" t="inlineStr">
-        <is>
-          <t>A Right That Exists on Paper, Exhibit 09</t>
-        </is>
-      </c>
-      <c r="P19" t="inlineStr">
-        <is>
-          <t>../compassionaterelease/index.html#from-statute-to-data</t>
+          <t>Small datasets, where a co-occurrence of two or three means nothing, and any reading of cause.</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>Chart form in common use; the example links to where this site uses it.</t>
+          <t>Counting coded themes is what Onwuegbuzie and Dickinson (2008) call quantitizing; their crossover displays chart the result.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>SPAN</t>
+          <t>CODEBK</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Span chart</t>
+          <t>Codebook table</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Ranges and thresholds</t>
+          <t>Matrices</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>One bar per case from its low value to its high, so the ranges line up.</t>
+          <t>Each code, its definition, and one passage that shows it.</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Number</t>
+          <t>Words;Nested</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Apart;Compare</t>
+          <t>Organised;Said</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Handful</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>Dozens</t>
-        </is>
-      </c>
-      <c r="J20" t="inlineStr">
-        <is>
-          <t>Helpful;Pattern</t>
-        </is>
-      </c>
-      <c r="K20" t="inlineStr">
-        <is>
-          <t>One;Two</t>
+          <t>One</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Passages</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>Thresholds that differ by case and sometimes depend on a condition, such as an age that depends on the sentence.</t>
+          <t>Making the coding auditable: a reader can check the rule against the example and argue with either.</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>Single values with no range; those want a dot plot.</t>
+          <t>Findings; it defines the instrument and shows no result.</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>A Right That Exists on Paper, Exhibit 03</t>
+          <t>A Right That Exists on Paper, Exhibit 09</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>../compassionaterelease/index.html#how-old-is-old-enough</t>
+          <t>../compassionaterelease/index.html#from-statute-to-data</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
@@ -2879,12 +2869,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>DOTS</t>
+          <t>SPAN</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Threshold dot plot</t>
+          <t>Span chart</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -2894,7 +2884,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Each case a dot on one scale, so clustering and outliers show at once.</t>
+          <t>One bar per case from its low value to its high, so the ranges line up.</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -2934,22 +2924,22 @@
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>A dozen or so statutory numbers on one scale, where the spread is the point.</t>
+          <t>Thresholds that differ by case and sometimes depend on a condition, such as an age that depends on the sentence.</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>Hundreds of values, which want a histogram, or values that cannot share a scale.</t>
+          <t>Single values with no range; those want a dot plot.</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>A Right That Exists on Paper, Exhibit 04</t>
+          <t>A Right That Exists on Paper, Exhibit 03</t>
         </is>
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>../compassionaterelease/index.html#how-long-is-terminal</t>
+          <t>../compassionaterelease/index.html#how-old-is-old-enough</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
@@ -2961,12 +2951,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>DUMB</t>
+          <t>DOTS</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Dumbbell</t>
+          <t>Threshold dot plot</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -2976,17 +2966,17 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Two dots per case joined by a line: before and after, or two codings of the same thing.</t>
+          <t>Each case a dot on one scale, so clustering and outliers show at once.</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Number;Sequence</t>
+          <t>Number</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Apart;Happened;Compare</t>
+          <t>Apart;Compare</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -3006,7 +2996,7 @@
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>Two</t>
+          <t>One;Two</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
@@ -3016,22 +3006,22 @@
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>A paired change, or a disagreement between two sources, case by case.</t>
+          <t>A dozen or so statutory numbers on one scale, where the spread is the point.</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>More than two points per case, or cases with only one.</t>
+          <t>Hundreds of values, which want a histogram, or values that cannot share a scale.</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>Maturity Gap, The Revolving Door</t>
+          <t>A Right That Exists on Paper, Exhibit 04</t>
         </is>
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>../countedwrong/index.html#the-revolving-door</t>
+          <t>../compassionaterelease/index.html#how-long-is-terminal</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
@@ -3043,37 +3033,37 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>TLINE</t>
+          <t>DUMB</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Vertical timeline</t>
+          <t>Dumbbell</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Time and process</t>
+          <t>Ranges and thresholds</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Dated events down the page, each with room for a phrase.</t>
+          <t>Two dots per case joined by a line: before and after, or two codings of the same thing.</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Sequence</t>
+          <t>Number;Sequence</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Happened</t>
+          <t>Apart;Happened;Compare</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>One</t>
+          <t>Handful</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -3081,34 +3071,39 @@
           <t>Dozens</t>
         </is>
       </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>Helpful;Pattern</t>
+        </is>
+      </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>One</t>
+          <t>Two</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>Phrases</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>One statute's or one program's history, when the events need words, because phrases need horizontal room.</t>
+          <t>A paired change, or a disagreement between two sources, case by case.</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>Comparing several histories; stack them and the labels collide.</t>
+          <t>More than two points per case, or cases with only one.</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>A Right That Exists on Paper, Exhibit 10</t>
+          <t>Maturity Gap, The Revolving Door</t>
         </is>
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>../compassionaterelease/index.html#one-state-thirty-years</t>
+          <t>../countedwrong/index.html#the-revolving-door</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">
@@ -3120,12 +3115,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>GANTT</t>
+          <t>TLINE</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Spans over time</t>
+          <t>Vertical timeline</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -3135,7 +3130,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>A bar per case from when it began to when it ended, stacked down the page.</t>
+          <t>Dated events down the page, each with room for a phrase.</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -3145,12 +3140,12 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Happened;Compare</t>
+          <t>Happened</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Handful</t>
+          <t>One</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -3158,41 +3153,51 @@
           <t>Dozens</t>
         </is>
       </c>
-      <c r="J24" t="inlineStr">
-        <is>
-          <t>Helpful;Pattern</t>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>One</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Phrases</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>When each policy was in force, or how long each case took, read against the others.</t>
+          <t>One statute's or one program's history, when the events need words, because phrases need horizontal room.</t>
         </is>
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>Events without duration, or cases whose dates are unknown.</t>
+          <t>Comparing several histories; stack them and the labels collide.</t>
+        </is>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>A Right That Exists on Paper, Exhibit 10</t>
+        </is>
+      </c>
+      <c r="P24" t="inlineStr">
+        <is>
+          <t>../compassionaterelease/index.html#one-state-thirty-years</t>
         </is>
       </c>
       <c r="Q24" t="inlineStr">
         <is>
-          <t>Henderson and Segal (2013) draw this as a chronological chart, one row per activity shaded when it was under way (their Figure 3.7).</t>
+          <t>Chart form in common use; the example links to where this site uses it.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>FLOW</t>
+          <t>GANTT</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Flowchart</t>
+          <t>Spans over time</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -3202,64 +3207,64 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Boxes and arrows: the steps, the decision points, and the paths cases take.</t>
+          <t>A bar per case from when it began to when it ended, stacked down the page.</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Process</t>
+          <t>Sequence</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Branch;Organised</t>
+          <t>Happened;Compare</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>One</t>
+          <t>Handful</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>Handful</t>
-        </is>
-      </c>
-      <c r="K25" t="inlineStr">
-        <is>
-          <t>One</t>
+          <t>Dozens</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>Helpful;Pattern</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>Phrases</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>A procedure as written, or as the people inside it describe it; the two drawn side by side is a finding.</t>
+          <t>When each policy was in force, or how long each case took, read against the others.</t>
         </is>
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>Counts of who went which way (a funnel or an alluvial does that), or a process with more than a dozen boxes.</t>
+          <t>Events without duration, or cases whose dates are unknown.</t>
         </is>
       </c>
       <c r="Q25" t="inlineStr">
         <is>
-          <t>Verdinelli and Scagnoli (2013), one of the nine display types in their review of three qualitative journals.</t>
+          <t>Henderson and Segal (2013) draw this as a chronological chart, one row per activity shaded when it was under way (their Figure 3.7).</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>DTREE</t>
+          <t>FLOW</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Decision tree</t>
+          <t>Flowchart</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -3269,7 +3274,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>The questions in the order they are asked, each answer leading to the next, ending in outcomes.</t>
+          <t>Boxes and arrows: the steps, the decision points, and the paths cases take.</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -3304,12 +3309,12 @@
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>Eligibility rules and screening logic, where readers want to trace their own case through.</t>
+          <t>A procedure as written, or as the people inside it describe it; the two drawn side by side is a finding.</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>Processes where the order of questions is not fixed, or outcomes that turn on judgment rather than rules.</t>
+          <t>Counts of who went which way (a funnel or an alluvial does that), or a process with more than a dozen boxes.</t>
         </is>
       </c>
       <c r="Q26" t="inlineStr">
@@ -3321,12 +3326,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>LADDER</t>
+          <t>DTREE</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Ladder (stage diagram)</t>
+          <t>Decision tree</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -3336,17 +3341,17 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Levels or stages stacked in order, each rung a phase the phenomenon passes through.</t>
+          <t>The questions in the order they are asked, each answer leading to the next, ending in outcomes.</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Process;Nested</t>
+          <t>Process</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Organised;Happened</t>
+          <t>Branch;Organised</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -3371,12 +3376,12 @@
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>A progression with named stages, such as how a court's use of data matures.</t>
+          <t>Eligibility rules and screening logic, where readers want to trace their own case through.</t>
         </is>
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>Anything that moves backward or skips stages; a ladder promises an order.</t>
+          <t>Processes where the order of questions is not fixed, or outcomes that turn on judgment rather than rules.</t>
         </is>
       </c>
       <c r="Q27" t="inlineStr">
@@ -3388,44 +3393,44 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>NET</t>
+          <t>LADDER</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Network (concept map)</t>
+          <t>Ladder (stage diagram)</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Relationships and structure</t>
+          <t>Time and process</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Nodes for themes or people and lines for the ties between them.</t>
+          <t>Levels or stages stacked in order, each rung a phase the phenomenon passes through.</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Relationships</t>
+          <t>Process;Nested</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Together;Organised</t>
+          <t>Organised;Happened</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
+          <t>One</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
           <t>Handful</t>
         </is>
       </c>
-      <c r="H28" t="inlineStr">
-        <is>
-          <t>Dozens</t>
-        </is>
-      </c>
       <c r="K28" t="inlineStr">
         <is>
           <t>One</t>
@@ -3438,29 +3443,29 @@
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>Showing how themes connect, or who talks to whom, when the ties are the finding.</t>
+          <t>A progression with named stages, such as how a court's use of data matures.</t>
         </is>
       </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t>A reader who needs to know how strong a tie is; lines of equal weight claim equal ties.</t>
+          <t>Anything that moves backward or skips stages; a ladder promises an order.</t>
         </is>
       </c>
       <c r="Q28" t="inlineStr">
         <is>
-          <t>Verdinelli and Scagnoli (2013), one of the nine display types in their review; Henderson and Segal (2013) draw the same thing as a thematic map; Miles, Huberman and Saldana's causal network is the explanatory version.</t>
+          <t>Verdinelli and Scagnoli (2013), one of the nine display types in their review of three qualitative journals.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>VENN</t>
+          <t>NET</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Modified Venn diagram</t>
+          <t>Network (concept map)</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -3470,12 +3475,12 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Overlapping circles for concepts that share ground, with the shared ground labelled.</t>
+          <t>Nodes for themes or people and lines for the ties between them.</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Relationships;Nested</t>
+          <t>Relationships</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -3485,19 +3490,19 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
+          <t>Handful</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>Dozens</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
           <t>One</t>
         </is>
       </c>
-      <c r="H29" t="inlineStr">
-        <is>
-          <t>Handful</t>
-        </is>
-      </c>
-      <c r="K29" t="inlineStr">
-        <is>
-          <t>One</t>
-        </is>
-      </c>
       <c r="L29" t="inlineStr">
         <is>
           <t>Phrases</t>
@@ -3505,29 +3510,29 @@
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>Two or three concepts whose overlap is the point.</t>
+          <t>Showing how themes connect, or who talks to whom, when the ties are the finding.</t>
         </is>
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>More than three sets, or any suggestion that the areas are proportional.</t>
+          <t>A reader who needs to know how strong a tie is; lines of equal weight claim equal ties.</t>
         </is>
       </c>
       <c r="Q29" t="inlineStr">
         <is>
-          <t>Verdinelli and Scagnoli (2013), one of the nine display types in their review of three qualitative journals.</t>
+          <t>Verdinelli and Scagnoli (2013), one of the nine display types in their review; Henderson and Segal (2013) draw the same thing as a thematic map; Miles, Huberman and Saldana's causal network is the explanatory version.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>TAX</t>
+          <t>VENN</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Taxonomy (tree diagram)</t>
+          <t>Modified Venn diagram</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -3537,17 +3542,17 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>The coding scheme as a tree: themes branching into subthemes.</t>
+          <t>Overlapping circles for concepts that share ground, with the shared ground labelled.</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Nested</t>
+          <t>Relationships;Nested</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Organised</t>
+          <t>Together;Organised</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -3557,7 +3562,7 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>Dozens</t>
+          <t>Handful</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
@@ -3572,12 +3577,12 @@
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>Showing the structure of the coding, so a reader can see what sits under what.</t>
+          <t>Two or three concepts whose overlap is the point.</t>
         </is>
       </c>
       <c r="N30" t="inlineStr">
         <is>
-          <t>Frequency or importance; a branch's position says nothing about its weight.</t>
+          <t>More than three sets, or any suggestion that the areas are proportional.</t>
         </is>
       </c>
       <c r="Q30" t="inlineStr">
@@ -3589,32 +3594,32 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>BOX</t>
+          <t>TAX</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Boxed display</t>
+          <t>Taxonomy (tree diagram)</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>The text itself</t>
+          <t>Relationships and structure</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>One passage, framed and set apart, so it is read as evidence rather than skimmed as prose.</t>
+          <t>The coding scheme as a tree: themes branching into subthemes.</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Words</t>
+          <t>Nested</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Said</t>
+          <t>Organised</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -3624,7 +3629,7 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>Handful</t>
+          <t>Dozens</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
@@ -3634,17 +3639,17 @@
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>Passages</t>
+          <t>Phrases</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>A single passage that says the thing better than any paraphrase.</t>
+          <t>Showing the structure of the coding, so a reader can see what sits under what.</t>
         </is>
       </c>
       <c r="N31" t="inlineStr">
         <is>
-          <t>Making a pattern claim; one box is one voice.</t>
+          <t>Frequency or importance; a branch's position says nothing about its weight.</t>
         </is>
       </c>
       <c r="Q31" t="inlineStr">
@@ -3656,12 +3661,12 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>QUOTES</t>
+          <t>BOX</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Exemplar quote cards</t>
+          <t>Boxed display</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -3671,7 +3676,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Several passages, each tagged with its code and its source, laid out as cards.</t>
+          <t>One passage, framed and set apart, so it is read as evidence rather than skimmed as prose.</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -3686,12 +3691,17 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
+          <t>One</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
           <t>Handful</t>
         </is>
       </c>
-      <c r="H32" t="inlineStr">
-        <is>
-          <t>Dozens</t>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>One</t>
         </is>
       </c>
       <c r="L32" t="inlineStr">
@@ -3701,29 +3711,29 @@
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>Showing the range inside a theme: the typical passage and the one that pushes against it.</t>
+          <t>A single passage that says the thing better than any paraphrase.</t>
         </is>
       </c>
       <c r="N32" t="inlineStr">
         <is>
-          <t>Prevalence; a wall of quotes reads as 'everyone said this' whether or not they did.</t>
+          <t>Making a pattern claim; one box is one voice.</t>
         </is>
       </c>
       <c r="Q32" t="inlineStr">
         <is>
-          <t>Illustrative excerpts are the traditional display of qualitative data in Henderson and Segal (2013); the cards add the code and the source to each.</t>
+          <t>Verdinelli and Scagnoli (2013), one of the nine display types in their review of three qualitative journals.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>EXCERPT</t>
+          <t>QUOTES</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Annotated excerpt</t>
+          <t>Exemplar quote cards</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -3733,32 +3743,27 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>A passage shown in full, with the coded spans highlighted and labelled in the margin.</t>
+          <t>Several passages, each tagged with its code and its source, laid out as cards.</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Words;Process</t>
+          <t>Words</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Said;Organised</t>
+          <t>Said</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>One</t>
+          <t>Handful</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>One</t>
-        </is>
-      </c>
-      <c r="K33" t="inlineStr">
-        <is>
-          <t>One</t>
+          <t>Dozens</t>
         </is>
       </c>
       <c r="L33" t="inlineStr">
@@ -3768,34 +3773,29 @@
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>Teaching the coding, or showing how a single document (a statute, a decision) was read.</t>
+          <t>Showing the range inside a theme: the typical passage and the one that pushes against it.</t>
         </is>
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t>More than one document; the point is depth, not breadth.</t>
+          <t>Prevalence; a wall of quotes reads as 'everyone said this' whether or not they did.</t>
         </is>
       </c>
       <c r="Q33" t="inlineStr">
         <is>
-          <t>Chart form in common use.</t>
-        </is>
-      </c>
-      <c r="T33" t="inlineStr">
-        <is>
-          <t>An annotated excerpt shows one document in depth; with {have}, the point is breadth, and a matrix carries that.</t>
+          <t>Illustrative excerpts are the traditional display of qualitative data in Henderson and Segal (2013); the cards add the code and the source to each.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>WTREE</t>
+          <t>EXCERPT</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Word tree</t>
+          <t>Annotated excerpt</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -3805,22 +3805,27 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>A phrase at the root, and every way the text continues from it branching to the right.</t>
+          <t>A passage shown in full, with the coded spans highlighted and labelled in the margin.</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Words;Relationships</t>
+          <t>Words;Process</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Together;Said</t>
+          <t>Said;Organised</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Dozens</t>
+          <t>One</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>One</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
@@ -3830,34 +3835,39 @@
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>Phrases</t>
+          <t>Passages</t>
         </is>
       </c>
       <c r="M34" t="inlineStr">
         <is>
-          <t>Exploring how a key term is used across a large corpus, in the speakers' own words.</t>
+          <t>Teaching the coding, or showing how a single document (a statute, a decision) was read.</t>
         </is>
       </c>
       <c r="N34" t="inlineStr">
         <is>
-          <t>Small corpora, where the tree is a few twigs, or a precise claim about frequency: size shows it roughly, and the rare branches are pruned.</t>
+          <t>More than one document; the point is depth, not breadth.</t>
         </is>
       </c>
       <c r="Q34" t="inlineStr">
         <is>
-          <t>Wattenberg and Viegas (2008), The Word Tree, an Interactive Visual Concordance; Henderson and Segal (2013), Visualizing Qualitative Data in Evaluation Research.</t>
+          <t>Chart form in common use.</t>
+        </is>
+      </c>
+      <c r="T34" t="inlineStr">
+        <is>
+          <t>An annotated excerpt shows one document in depth; with {have}, the point is breadth, and a matrix carries that.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>CLOUD</t>
+          <t>WTREE</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Word cloud</t>
+          <t>Word tree</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -3867,27 +3877,22 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Words sized by how often they appear, scattered on the page. Kept here so the page can say why it rarely fits.</t>
+          <t>A phrase at the root, and every way the text continues from it branching to the right.</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Words</t>
+          <t>Words;Relationships</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Common</t>
+          <t>Together;Said</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Many</t>
-        </is>
-      </c>
-      <c r="I35" t="inlineStr">
-        <is>
-          <t>Census;Designed</t>
+          <t>Dozens</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
@@ -3902,76 +3907,66 @@
       </c>
       <c r="M35" t="inlineStr">
         <is>
-          <t>A decorative opener, labelled as one, over a corpus large enough that word frequency means something.</t>
+          <t>Exploring how a key term is used across a large corpus, in the speakers' own words.</t>
         </is>
       </c>
       <c r="N35" t="inlineStr">
         <is>
-          <t>Almost everything else. How often a word appears is not how often a meaning does, size is read imprecisely, and the layout is random, so the figure answers a question nobody asked.</t>
+          <t>Small corpora, where the tree is a few twigs, or a precise claim about frequency: size shows it roughly, and the rare branches are pruned.</t>
         </is>
       </c>
       <c r="Q35" t="inlineStr">
         <is>
-          <t>Henderson and Segal (2013), Visualizing Qualitative Data in Evaluation Research.</t>
-        </is>
-      </c>
-      <c r="R35" t="inlineStr">
-        <is>
-          <t>A word cloud is a count of words, and from {have} it will be read as a count of meanings; neither reading holds.</t>
-        </is>
-      </c>
-      <c r="S35" t="inlineStr">
-        <is>
-          <t>A word cloud answers 'which words appear most', which is not {have}, and how often a word appears is not how often a meaning does.</t>
+          <t>Wattenberg and Viegas (2008), The Word Tree, an Interactive Visual Concordance; Henderson and Segal (2013), Visualizing Qualitative Data in Evaluation Research.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>DIAG</t>
+          <t>CLOUD</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Explanatory diagram</t>
+          <t>Word cloud</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Metaphor and illustration</t>
+          <t>The text itself</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>A drawing of the idea itself: the curve, the gap, the mechanism, with no data axis.</t>
+          <t>Words sized by how often they appear, scattered on the page. Kept here so the page can say why it rarely fits.</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Process;Relationships;Nested</t>
+          <t>Words</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Organised</t>
+          <t>Common</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
+          <t>Many</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>Census;Designed</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
           <t>One</t>
         </is>
       </c>
-      <c r="H36" t="inlineStr">
-        <is>
-          <t>One</t>
-        </is>
-      </c>
-      <c r="K36" t="inlineStr">
-        <is>
-          <t>One</t>
-        </is>
-      </c>
       <c r="L36" t="inlineStr">
         <is>
           <t>Phrases</t>
@@ -3979,44 +3974,39 @@
       </c>
       <c r="M36" t="inlineStr">
         <is>
-          <t>Setting up a frame the data charts then test, drawn once and referred back to.</t>
+          <t>A decorative opener, labelled as one, over a corpus large enough that word frequency means something.</t>
         </is>
       </c>
       <c r="N36" t="inlineStr">
         <is>
-          <t>Standing in for evidence; a diagram shows what you believe, and the charts after it have to earn it.</t>
-        </is>
-      </c>
-      <c r="O36" t="inlineStr">
-        <is>
-          <t>Maturity Gap, The Frame</t>
-        </is>
-      </c>
-      <c r="P36" t="inlineStr">
-        <is>
-          <t>../countedwrong/index.html#the-frame</t>
+          <t>Almost everything else. How often a word appears is not how often a meaning does, size is read imprecisely, and the layout is random, so the figure answers a question nobody asked.</t>
         </is>
       </c>
       <c r="Q36" t="inlineStr">
         <is>
-          <t>Chart form in common use; the example links to where this site uses it.</t>
-        </is>
-      </c>
-      <c r="T36" t="inlineStr">
-        <is>
-          <t>An explanatory diagram draws the idea, not the cases, so {have} is data waiting for a chart, with the diagram as its frame.</t>
+          <t>Henderson and Segal (2013), Visualizing Qualitative Data in Evaluation Research.</t>
+        </is>
+      </c>
+      <c r="R36" t="inlineStr">
+        <is>
+          <t>A word cloud is a count of words, and from {have} it will be read as a count of meanings; neither reading holds.</t>
+        </is>
+      </c>
+      <c r="S36" t="inlineStr">
+        <is>
+          <t>A word cloud answers 'which words appear most', which is not {have}, and how often a word appears is not how often a meaning does.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>META</t>
+          <t>DIAG</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Metaphorical display</t>
+          <t>Explanatory diagram</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -4026,17 +4016,17 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>The themes arranged as something else: a tree, a river, a house, whatever the data suggest.</t>
+          <t>A drawing of the idea itself: the curve, the gap, the mechanism, with no data axis.</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Nested;Relationships</t>
+          <t>Process;Relationships;Nested</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Organised;Together</t>
+          <t>Organised</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -4046,7 +4036,7 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>Handful</t>
+          <t>One</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
@@ -4061,29 +4051,44 @@
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>A public or participant audience, when the structure of the findings maps cleanly onto a familiar image.</t>
+          <t>Setting up a frame the data charts then test, drawn once and referred back to.</t>
         </is>
       </c>
       <c r="N37" t="inlineStr">
         <is>
-          <t>A technical reader, or any metaphor the data have to be bent to fit.</t>
+          <t>Standing in for evidence; a diagram shows what you believe, and the charts after it have to earn it.</t>
+        </is>
+      </c>
+      <c r="O37" t="inlineStr">
+        <is>
+          <t>Maturity Gap, The Frame</t>
+        </is>
+      </c>
+      <c r="P37" t="inlineStr">
+        <is>
+          <t>../countedwrong/index.html#the-frame</t>
         </is>
       </c>
       <c r="Q37" t="inlineStr">
         <is>
-          <t>Verdinelli and Scagnoli (2013), one of the nine display types in their review of three qualitative journals.</t>
+          <t>Chart form in common use; the example links to where this site uses it.</t>
+        </is>
+      </c>
+      <c r="T37" t="inlineStr">
+        <is>
+          <t>An explanatory diagram draws the idea, not the cases, so {have} is data waiting for a chart, with the diagram as its frame.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>JOURNEY</t>
+          <t>META</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Journey map</t>
+          <t>Metaphorical display</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -4093,17 +4098,17 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>One case's path through the system, step by step, with what happened and how it was experienced at each.</t>
+          <t>The themes arranged as something else: a tree, a river, a house, whatever the data suggest.</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Process;Words;Sequence</t>
+          <t>Nested;Relationships</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Happened;Said</t>
+          <t>Organised;Together</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -4123,95 +4128,153 @@
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>Passages</t>
+          <t>Phrases</t>
         </is>
       </c>
       <c r="M38" t="inlineStr">
         <is>
-          <t>Making a procedure concrete through one person's or one case's passage, with their words at each step.</t>
+          <t>A public or participant audience, when the structure of the findings maps cleanly onto a familiar image.</t>
         </is>
       </c>
       <c r="N38" t="inlineStr">
         <is>
-          <t>Claiming the path is typical; one journey is one journey unless the cases behind it are shown.</t>
+          <t>A technical reader, or any metaphor the data have to be bent to fit.</t>
         </is>
       </c>
       <c r="Q38" t="inlineStr">
         <is>
-          <t>Added from practice (2026).</t>
+          <t>Verdinelli and Scagnoli (2013), one of the nine display types in their review of three qualitative journals.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
+          <t>JOURNEY</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Journey map</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Metaphor and illustration</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>One case's path through the system, step by step, with what happened and how it was experienced at each.</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Process;Words;Sequence</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>Happened;Said</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>One</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>Handful</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>One</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>Passages</t>
+        </is>
+      </c>
+      <c r="M39" t="inlineStr">
+        <is>
+          <t>Making a procedure concrete through one person's or one case's passage, with their words at each step.</t>
+        </is>
+      </c>
+      <c r="N39" t="inlineStr">
+        <is>
+          <t>Claiming the path is typical; one journey is one journey unless the cases behind it are shown.</t>
+        </is>
+      </c>
+      <c r="Q39" t="inlineStr">
+        <is>
+          <t>Added from practice (2026).</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
           <t>CHORO</t>
         </is>
       </c>
-      <c r="B39" t="inlineStr">
+      <c r="B40" t="inlineStr">
         <is>
           <t>Choropleth map (shaded areas)</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr">
+      <c r="C40" t="inlineStr">
         <is>
           <t>Places and maps</t>
         </is>
       </c>
-      <c r="D39" t="inlineStr">
+      <c r="D40" t="inlineStr">
         <is>
           <t>Each place on its own outline, shaded by a value or marked for a feature.</t>
         </is>
       </c>
-      <c r="E39" t="inlineStr">
+      <c r="E40" t="inlineStr">
         <is>
           <t>Places</t>
         </is>
       </c>
-      <c r="F39" t="inlineStr">
+      <c r="F40" t="inlineStr">
         <is>
           <t>Compare;Common</t>
         </is>
       </c>
-      <c r="G39" t="inlineStr">
+      <c r="G40" t="inlineStr">
         <is>
           <t>Handful</t>
         </is>
       </c>
-      <c r="H39" t="inlineStr"/>
-      <c r="I39" t="inlineStr"/>
-      <c r="J39" t="inlineStr">
+      <c r="J40" t="inlineStr">
         <is>
           <t>Helpful;Pattern</t>
         </is>
       </c>
-      <c r="K39" t="inlineStr"/>
-      <c r="L39" t="inlineStr">
+      <c r="L40" t="inlineStr">
         <is>
           <t>Pattern</t>
         </is>
       </c>
-      <c r="M39" t="inlineStr">
+      <c r="M40" t="inlineStr">
         <is>
           <t>Cases that are places, when where a feature sits is part of the finding: which circuits named transportation, which states require a diagnosis, one map per feature if there are several.</t>
         </is>
       </c>
-      <c r="N39" t="inlineStr">
+      <c r="N40" t="inlineStr">
         <is>
           <t>Reading size from area. Large rural units fill the eye while a city of a million is a speck, so label the small ones, add an inset, or let the map carry the geography and a heatmap carry the comparison.</t>
         </is>
       </c>
-      <c r="O39" t="inlineStr"/>
-      <c r="P39" t="inlineStr"/>
-      <c r="Q39" t="inlineStr">
+      <c r="Q40" t="inlineStr">
         <is>
           <t>Chart form in common use, the thematic map's workhorse; cartographic sources to follow the visualization-literature rescan.</t>
         </is>
       </c>
-      <c r="R39" t="inlineStr"/>
-      <c r="S39" t="inlineStr"/>
-      <c r="T39" t="inlineStr"/>
-      <c r="U39" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Pickers: numeric case-count chips; "Tap or click" hint
The qualitative picker's case chip now uses numbers that match the
units question's own ranges ("1 to 9 cases", "2 to 50 cases", "10 or
more cases", "more than 50 cases"), replacing word ranges such as "a
few to dozens cases". New Copy key scale_over, checked by 5c.

All three pickers' results-bar hint now reads "Tap or click ...",
since most visitors arrive on a phone.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0191t4cG3m6aQycW3EiNAUvs
</commit_message>
<xml_diff>
--- a/qualpicker/data/qualitative_displays.xlsx
+++ b/qualpicker/data/qualitative_displays.xlsx
@@ -4287,7 +4287,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B56"/>
+  <dimension ref="A1:B57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -4542,7 +4542,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Click any display for the detail.</t>
+          <t>Tap or click any display for the detail.</t>
         </is>
       </c>
     </row>
@@ -4801,166 +4801,178 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>reason_shape_ok</t>
+          <t>scale_over</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>{display} works from {needed}, and what you have is {have}.</t>
+          <t>more than 50 cases</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>short_shape_ok</t>
+          <t>reason_shape_ok</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Different evidence</t>
+          <t>{display} works from {needed}, and what you have is {have}.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>reason_question_ok</t>
+          <t>short_shape_ok</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>{display} answers {needed}, not {have}.</t>
+          <t>Different evidence</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>short_question_ok</t>
+          <t>reason_question_ok</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Different question</t>
+          <t>{display} answers {needed}, not {have}.</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>reason_units_min</t>
+          <t>short_question_ok</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>{display} needs {needed} to read as a pattern, and with {have} it would show noise, or dress a few cases as a trend.</t>
+          <t>Different question</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>short_units_min</t>
+          <t>reason_units_min</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Too few cases</t>
+          <t>{display} needs {needed} to read as a pattern, and with {have} it would show noise, or dress a few cases as a trend.</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>reason_units_max</t>
+          <t>short_units_min</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>{display} stops being readable past {needed}; with {have}, the labels and cells outnumber what a reader can hold.</t>
+          <t>Too few cases</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>short_units_max</t>
+          <t>reason_units_max</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Too many cases</t>
+          <t>{display} stops being readable past {needed}; with {have}, the labels and cells outnumber what a reader can hold.</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>reason_counting_ok</t>
+          <t>short_units_max</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>{display} reads as a count, and a reader will take a count as how common something is; that holds for {needed}, not for {have}.</t>
+          <t>Too many cases</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>short_counting_ok</t>
+          <t>reason_counting_ok</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Count would overreach</t>
+          <t>{display} reads as a count, and a reader will take a count as how common something is; that holds for {needed}, not for {have}.</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>reason_words_ok</t>
+          <t>short_counting_ok</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>{display} shows the pattern and not the passages, so when the quotes carry the evidence it needs the text beside it, or a form that shows the words.</t>
+          <t>Count would overreach</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>short_words_ok</t>
+          <t>reason_words_ok</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Pair with the text</t>
+          <t>{display} shows the pattern and not the passages, so when the quotes carry the evidence it needs the text beside it, or a form that shows the words.</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>reason_groups_ok</t>
+          <t>short_words_ok</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>{display} is built for {needed}; with {have} there is either nothing to compare or too much in one panel.</t>
+          <t>Pair with the text</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
+          <t>reason_groups_ok</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>{display} is built for {needed}; with {have} there is either nothing to compare or too much in one panel.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
           <t>short_groups_ok</t>
         </is>
       </c>
-      <c r="B56" t="inlineStr">
+      <c r="B57" t="inlineStr">
         <is>
           <t>Different comparison</t>
         </is>

</xml_diff>